<commit_message>
Edited Excell.. Edited backend..
</commit_message>
<xml_diff>
--- a/Kuka/Kuka_Promenne.xlsx
+++ b/Kuka/Kuka_Promenne.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Disk\Vysoka skola\Magisterske_studium\3_semester\Project_AdvancedPianistRobot\AdvancedPianistRobot\Kuka\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47094D5F-1BBD-489D-897F-B76EAE840319}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BC91110-EE4B-46BA-9B53-FEFF182693ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{63C010F2-5D75-486A-A0FE-7CCEE5BD46F5}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="26">
   <si>
     <t>Proměnná</t>
   </si>
@@ -44,12 +44,6 @@
     <t>FeedBack Proměnné</t>
   </si>
   <si>
-    <t>PyStartShadowing</t>
-  </si>
-  <si>
-    <t>PyStopShadowing</t>
-  </si>
-  <si>
     <t>PyMAX_VOLUME</t>
   </si>
   <si>
@@ -111,6 +105,15 @@
   </si>
   <si>
     <t>PyNoteDuration</t>
+  </si>
+  <si>
+    <t>PyNotePlayed</t>
+  </si>
+  <si>
+    <t>PyShadow</t>
+  </si>
+  <si>
+    <t>PyShadowFb</t>
   </si>
 </sst>
 </file>
@@ -191,16 +194,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
@@ -545,7 +547,7 @@
   <cols>
     <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.85546875" customWidth="1"/>
-    <col min="5" max="5" width="19" customWidth="1"/>
+    <col min="5" max="5" width="20.42578125" customWidth="1"/>
     <col min="8" max="8" width="15.28515625" customWidth="1"/>
     <col min="9" max="9" width="21.28515625" customWidth="1"/>
     <col min="10" max="10" width="11.5703125" customWidth="1"/>
@@ -553,160 +555,160 @@
   <sheetData>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D4" s="5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
       <c r="H4" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I4" s="5"/>
       <c r="J4" s="5"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="F5" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="H5" s="6" t="s">
+      <c r="F5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="J5" s="6" t="s">
-        <v>9</v>
+      <c r="J5" s="4" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D6" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3" t="s">
-        <v>10</v>
+      <c r="D6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>8</v>
       </c>
       <c r="H6" t="s">
+        <v>14</v>
+      </c>
+      <c r="J6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="3"/>
+      <c r="B7" t="s">
         <v>16</v>
       </c>
-      <c r="J6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
-      <c r="B7" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3" t="s">
-        <v>11</v>
+      <c r="D7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3" t="s">
+      <c r="F9" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D12" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D13" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D14" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D15" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D16" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D18" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="D9" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D10" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D12" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D13" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D14" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D15" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D16" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4" t="s">
+      <c r="E18" s="3"/>
+      <c r="F18" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D19" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="18" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D18" s="4" t="s">
+      <c r="E19" s="3"/>
+      <c r="F19" s="3" t="s">
         <v>12</v>
-      </c>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D19" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Code in monitor.. on pianist.. and other edits
</commit_message>
<xml_diff>
--- a/Kuka/Kuka_Promenne.xlsx
+++ b/Kuka/Kuka_Promenne.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Disk\Vysoka skola\Magisterske_studium\3_semester\Project_AdvancedPianistRobot\AdvancedPianistRobot\Kuka\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BC91110-EE4B-46BA-9B53-FEFF182693ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED1D908A-56D3-4661-A39A-A645BD89345E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{63C010F2-5D75-486A-A0FE-7CCEE5BD46F5}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" xr2:uid="{63C010F2-5D75-486A-A0FE-7CCEE5BD46F5}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="27">
   <si>
     <t>Proměnná</t>
   </si>
@@ -114,6 +114,9 @@
   </si>
   <si>
     <t>PyShadowFb</t>
+  </si>
+  <si>
+    <t>PyKey</t>
   </si>
 </sst>
 </file>
@@ -542,7 +545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CC30636-6410-451D-BD1C-8D7430EFCB92}">
-  <dimension ref="A4:J19"/>
+  <dimension ref="A4:J20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
@@ -648,18 +651,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D12" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3" t="s">
-        <v>8</v>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D13" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3" t="s">
@@ -668,7 +671,7 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D14" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3" t="s">
@@ -677,7 +680,7 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D15" s="3" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3" t="s">
@@ -686,28 +689,37 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D16" s="3" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D17" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3" t="s">
         <v>9</v>
-      </c>
-    </row>
-    <row r="18" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D18" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="19" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D19" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D20" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added files from Rpi... Added Rpi diagnostics to backend.. and working paralel connect to kuka
</commit_message>
<xml_diff>
--- a/Kuka/Kuka_Promenne.xlsx
+++ b/Kuka/Kuka_Promenne.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AdvancedPianistRobot\Kuka\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Disk\Vysoka skola\Magisterske_studium\3_semester\Project_AdvancedPianistRobot\AdvancedPianistRobot\Kuka\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6EB9397-840E-4D2D-A5CF-71808955D385}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{412D31A8-BDDE-4C7D-942D-7502A381F9F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{63C010F2-5D75-486A-A0FE-7CCEE5BD46F5}"/>
   </bookViews>
@@ -554,30 +554,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CC30636-6410-451D-BD1C-8D7430EFCB92}">
-  <dimension ref="A4:J20"/>
+  <dimension ref="A4:K20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.85546875" customWidth="1"/>
     <col min="5" max="5" width="20.42578125" customWidth="1"/>
-    <col min="8" max="8" width="15.28515625" customWidth="1"/>
-    <col min="9" max="9" width="21.28515625" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" customWidth="1"/>
+    <col min="9" max="9" width="15.28515625" customWidth="1"/>
+    <col min="10" max="10" width="21.28515625" customWidth="1"/>
+    <col min="11" max="11" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D4" s="5" t="s">
         <v>18</v>
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
-      <c r="H4" s="5" t="s">
+      <c r="I4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="I4" s="5"/>
       <c r="J4" s="5"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K4" s="5"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D5" s="4" t="s">
         <v>0</v>
       </c>
@@ -587,20 +587,20 @@
       <c r="F5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="I5" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="J5" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="K5" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D6" s="2" t="s">
         <v>24</v>
       </c>
@@ -610,17 +610,17 @@
       <c r="F6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>14</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" t="s">
         <v>16</v>
@@ -632,11 +632,11 @@
       <c r="F7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" t="s">
         <v>17</v>
@@ -648,11 +648,11 @@
       <c r="F8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D9" s="2" t="s">
         <v>20</v>
       </c>
@@ -662,11 +662,11 @@
       <c r="F9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D10" s="2" t="s">
         <v>23</v>
       </c>
@@ -674,11 +674,11 @@
       <c r="F10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D11" s="2" t="s">
         <v>26</v>
       </c>
@@ -686,8 +686,9 @@
       <c r="F11" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G11" s="2"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D13" s="3" t="s">
         <v>3</v>
       </c>
@@ -695,11 +696,11 @@
       <c r="F13" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D14" s="3" t="s">
         <v>4</v>
       </c>
@@ -707,11 +708,11 @@
       <c r="F14" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D15" s="3" t="s">
         <v>5</v>
       </c>
@@ -719,11 +720,11 @@
       <c r="F15" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D16" s="3" t="s">
         <v>2</v>
       </c>
@@ -731,7 +732,7 @@
       <c r="F16" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16" s="3" t="s">
         <v>28</v>
       </c>
     </row>
@@ -743,7 +744,7 @@
       <c r="F17" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="3" t="s">
         <v>28</v>
       </c>
     </row>
@@ -755,7 +756,7 @@
       <c r="F19" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G19" s="3" t="s">
         <v>28</v>
       </c>
     </row>
@@ -767,14 +768,14 @@
       <c r="F20" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G20" s="3" t="s">
         <v>28</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="D4:F4"/>
-    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="I4:K4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Mnogo vecí Xd.. povetšinou s websocketem
</commit_message>
<xml_diff>
--- a/Kuka/Kuka_Promenne.xlsx
+++ b/Kuka/Kuka_Promenne.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Disk\Vysoka skola\Magisterske_studium\3_semester\Project_AdvancedPianistRobot\AdvancedPianistRobot\Kuka\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{412D31A8-BDDE-4C7D-942D-7502A381F9F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCA960FF-FC0E-4D15-B2B5-8FFCE6781361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{63C010F2-5D75-486A-A0FE-7CCEE5BD46F5}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" xr2:uid="{63C010F2-5D75-486A-A0FE-7CCEE5BD46F5}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="31">
   <si>
     <t>Proměnná</t>
   </si>
@@ -126,6 +126,9 @@
   </si>
   <si>
     <t>Int</t>
+  </si>
+  <si>
+    <t>PyPlayingSong</t>
   </si>
 </sst>
 </file>
@@ -554,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CC30636-6410-451D-BD1C-8D7430EFCB92}">
-  <dimension ref="A4:K20"/>
+  <dimension ref="A4:K22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
@@ -688,33 +691,21 @@
       </c>
       <c r="G11" s="2"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D13" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D14" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G14" s="3" t="s">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D12" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D15" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3" t="s">
@@ -726,7 +717,7 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D16" s="3" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3" t="s">
@@ -738,37 +729,61 @@
     </row>
     <row r="17" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D17" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G17" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D18" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G18" s="3" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="19" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D19" s="3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D21" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G19" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="20" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D20" s="3" t="s">
+      <c r="G21" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D22" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3" t="s">
+      <c r="E22" s="3"/>
+      <c r="F22" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="G22" s="3" t="s">
         <v>28</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Tested on robot aaa fungujeeee
</commit_message>
<xml_diff>
--- a/Kuka/Kuka_Promenne.xlsx
+++ b/Kuka/Kuka_Promenne.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Disk\Vysoka skola\Magisterske_studium\3_semester\Project_AdvancedPianistRobot\AdvancedPianistRobot\Kuka\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCA960FF-FC0E-4D15-B2B5-8FFCE6781361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80E00793-0592-45F4-A7D0-277CB55707E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" xr2:uid="{63C010F2-5D75-486A-A0FE-7CCEE5BD46F5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{63C010F2-5D75-486A-A0FE-7CCEE5BD46F5}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -162,7 +162,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -184,6 +184,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -209,12 +215,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -569,16 +576,16 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="I4" s="5" t="s">
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="I4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D5" s="4" t="s">
@@ -628,14 +635,14 @@
       <c r="B7" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2" t="s">
+      <c r="E7" s="5"/>
+      <c r="F7" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="5" t="s">
         <v>29</v>
       </c>
     </row>
@@ -659,7 +666,7 @@
       <c r="D9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F9" s="2" t="s">
@@ -670,14 +677,14 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2" t="s">
+      <c r="E10" s="5"/>
+      <c r="F10" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="5" t="s">
         <v>29</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Backend functional edits in frontend
</commit_message>
<xml_diff>
--- a/Kuka/Kuka_Promenne.xlsx
+++ b/Kuka/Kuka_Promenne.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Disk\Vysoka skola\Magisterske_studium\3_semester\Project_AdvancedPianistRobot\AdvancedPianistRobot\Kuka\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80E00793-0592-45F4-A7D0-277CB55707E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63F8F31D-05CD-466C-8DF2-96EFA77B13B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{63C010F2-5D75-486A-A0FE-7CCEE5BD46F5}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="32">
   <si>
     <t>Proměnná</t>
   </si>
@@ -129,6 +129,9 @@
   </si>
   <si>
     <t>PyPlayingSong</t>
+  </si>
+  <si>
+    <t>PySongNumber</t>
   </si>
 </sst>
 </file>
@@ -710,6 +713,17 @@
         <v>28</v>
       </c>
     </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D15" s="3" t="s">
         <v>3</v>

</xml_diff>